<commit_message>
Fianlização do Resultado Macro.
</commit_message>
<xml_diff>
--- a/dados/macro_final.xlsx
+++ b/dados/macro_final.xlsx
@@ -5,16 +5,17 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\victo\Documents\dev_2026\gd_impacta_mg\dados\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\desenvolvimentos\apps\gd_impacta_mg\dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B05B1F5-AFB9-4AB5-9212-0183958B498F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3265AB1-F485-451C-8E5A-6525C8C59EAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="812" firstSheet="1" activeTab="1" xr2:uid="{6BD6CDAF-41BA-4A42-8104-E0BB62F5B055}"/>
+    <workbookView xWindow="25695" yWindow="10440" windowWidth="26010" windowHeight="10545" tabRatio="812" activeTab="2" xr2:uid="{6BD6CDAF-41BA-4A42-8104-E0BB62F5B055}"/>
   </bookViews>
   <sheets>
     <sheet name="Agregados Macroeconômicos" sheetId="1" r:id="rId1"/>
     <sheet name="Produção Setorial" sheetId="2" r:id="rId2"/>
+    <sheet name="ICMS Setorial" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="22">
   <si>
     <t>variavel</t>
   </si>
@@ -112,10 +113,26 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -138,13 +155,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Moeda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -478,16 +498,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E34B4D21-0349-4A2C-99F1-0686022FD50F}">
   <dimension ref="A1:E17"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.86328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="7" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.73046875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.3984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -504,7 +524,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -521,7 +541,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -538,7 +558,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -555,7 +575,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -572,7 +592,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -589,7 +609,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -606,7 +626,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -623,7 +643,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -640,7 +660,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -657,7 +677,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>5</v>
       </c>
@@ -674,7 +694,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>6</v>
       </c>
@@ -691,7 +711,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>21</v>
       </c>
@@ -708,7 +728,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>7</v>
       </c>
@@ -725,7 +745,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>8</v>
       </c>
@@ -742,7 +762,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>9</v>
       </c>
@@ -759,7 +779,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>10</v>
       </c>
@@ -784,15 +804,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E19BC87-F2ED-435D-A7B4-31548BF1A397}">
   <dimension ref="A1:D13"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.86328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.1328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -806,7 +826,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -820,7 +840,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -834,7 +854,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -848,7 +868,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>18</v>
       </c>
@@ -862,7 +882,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -876,7 +896,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>20</v>
       </c>
@@ -890,7 +910,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -904,7 +924,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -918,7 +938,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>17</v>
       </c>
@@ -932,7 +952,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>18</v>
       </c>
@@ -946,7 +966,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -960,7 +980,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>20</v>
       </c>
@@ -977,4 +997,202 @@
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{705C5CE6-3297-4960-852C-11C20C32F211}">
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="1">
+        <v>1641.8455060380932</v>
+      </c>
+      <c r="D2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="1">
+        <v>9793.9936734852326</v>
+      </c>
+      <c r="D3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="1">
+        <v>109614.11780827655</v>
+      </c>
+      <c r="D4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="1">
+        <v>8471.4632975676868</v>
+      </c>
+      <c r="D5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="1">
+        <v>95431.921069947828</v>
+      </c>
+      <c r="D6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="1">
+        <v>1895.7817602001583</v>
+      </c>
+      <c r="D7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="1">
+        <v>1723.0793831474577</v>
+      </c>
+      <c r="D8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="1">
+        <v>10785.057413165567</v>
+      </c>
+      <c r="D9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="1">
+        <v>116901.02887996256</v>
+      </c>
+      <c r="D10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" s="1">
+        <v>8763.8102633303388</v>
+      </c>
+      <c r="D11" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" s="1">
+        <v>108107.4089178436</v>
+      </c>
+      <c r="D12" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" s="1">
+        <v>2040.0024775608281</v>
+      </c>
+      <c r="D13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
 </file>
</xml_diff>